<commit_message>
Agregue comentarios en todos los codigos con la estructura del proceso, y cree funcion procesar_diferencias
</commit_message>
<xml_diff>
--- a/app/Archivos/Template/Template_HRC_Cenco.xlsx
+++ b/app/Archivos/Template/Template_HRC_Cenco.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I315"/>
+  <dimension ref="A1:I314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>9168890610.360001</v>
+        <v>9168890459</v>
       </c>
     </row>
     <row r="8">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>9168890610.360001</v>
+        <v>9168890459</v>
       </c>
     </row>
     <row r="9"/>
@@ -626,7 +626,7 @@
     <row r="19">
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="20">
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -668,7 +668,7 @@
     <row r="21">
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
@@ -689,7 +689,7 @@
     <row r="22">
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
@@ -710,7 +710,7 @@
     <row r="23">
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -731,7 +731,7 @@
     <row r="24">
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
@@ -752,7 +752,7 @@
     <row r="25">
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -773,7 +773,7 @@
     <row r="26">
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
@@ -794,7 +794,7 @@
     <row r="27">
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
@@ -815,7 +815,7 @@
     <row r="28">
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
@@ -836,7 +836,7 @@
     <row r="29">
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="30">
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
@@ -878,7 +878,7 @@
     <row r="31">
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -899,7 +899,7 @@
     <row r="32">
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -920,7 +920,7 @@
     <row r="33">
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -941,7 +941,7 @@
     <row r="34">
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
@@ -962,7 +962,7 @@
     <row r="35">
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="36">
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
@@ -1004,7 +1004,7 @@
     <row r="37">
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
@@ -1025,7 +1025,7 @@
     <row r="38">
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
@@ -1046,7 +1046,7 @@
     <row r="39">
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="40">
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="41">
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
@@ -1109,7 +1109,7 @@
     <row r="42">
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
@@ -1130,7 +1130,7 @@
     <row r="43">
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
@@ -1151,7 +1151,7 @@
     <row r="44">
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="45">
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
@@ -1193,7 +1193,7 @@
     <row r="46">
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
@@ -1214,7 +1214,7 @@
     <row r="47">
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
@@ -1256,7 +1256,7 @@
     <row r="49">
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="50">
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
@@ -1298,7 +1298,7 @@
     <row r="51">
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
@@ -1319,7 +1319,7 @@
     <row r="52">
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
@@ -1340,7 +1340,7 @@
     <row r="53">
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
@@ -1361,7 +1361,7 @@
     <row r="54">
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
@@ -1382,7 +1382,7 @@
     <row r="55">
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
@@ -1403,7 +1403,7 @@
     <row r="56">
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
@@ -1424,7 +1424,7 @@
     <row r="57">
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
@@ -1445,7 +1445,7 @@
     <row r="58">
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
@@ -1466,7 +1466,7 @@
     <row r="59">
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="60">
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
@@ -1508,7 +1508,7 @@
     <row r="61">
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
@@ -1529,7 +1529,7 @@
     <row r="62">
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
@@ -1550,7 +1550,7 @@
     <row r="63">
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
@@ -1571,7 +1571,7 @@
     <row r="64">
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
@@ -1592,7 +1592,7 @@
     <row r="65">
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
@@ -1613,7 +1613,7 @@
     <row r="66">
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
@@ -1634,7 +1634,7 @@
     <row r="67">
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
@@ -1655,7 +1655,7 @@
     <row r="68">
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
@@ -1676,7 +1676,7 @@
     <row r="69">
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="70">
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
@@ -1718,7 +1718,7 @@
     <row r="71">
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="72">
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
@@ -1760,7 +1760,7 @@
     <row r="73">
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
@@ -1781,7 +1781,7 @@
     <row r="74">
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
@@ -1802,7 +1802,7 @@
     <row r="75">
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
@@ -1823,7 +1823,7 @@
     <row r="76">
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
@@ -1844,7 +1844,7 @@
     <row r="77">
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
@@ -1865,7 +1865,7 @@
     <row r="78">
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
@@ -1886,7 +1886,7 @@
     <row r="79">
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="80">
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
@@ -1928,7 +1928,7 @@
     <row r="81">
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
@@ -1949,7 +1949,7 @@
     <row r="82">
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
@@ -1970,7 +1970,7 @@
     <row r="83">
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
@@ -1991,7 +1991,7 @@
     <row r="84">
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
@@ -2012,7 +2012,7 @@
     <row r="85">
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
@@ -2033,7 +2033,7 @@
     <row r="86">
       <c r="C86" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
@@ -2054,7 +2054,7 @@
     <row r="87">
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
@@ -2075,7 +2075,7 @@
     <row r="88">
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <row r="89">
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="90">
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
@@ -2138,7 +2138,7 @@
     <row r="91">
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
@@ -2159,7 +2159,7 @@
     <row r="92">
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
@@ -2180,7 +2180,7 @@
     <row r="93">
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
@@ -2201,7 +2201,7 @@
     <row r="94">
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
@@ -2222,7 +2222,7 @@
     <row r="95">
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
@@ -2243,7 +2243,7 @@
     <row r="96">
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="97">
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
@@ -2285,7 +2285,7 @@
     <row r="98">
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="99">
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="100">
       <c r="C100" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
@@ -2348,7 +2348,7 @@
     <row r="101">
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
@@ -2369,7 +2369,7 @@
     <row r="102">
       <c r="C102" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
@@ -2390,7 +2390,7 @@
     <row r="103">
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
@@ -2411,7 +2411,7 @@
     <row r="104">
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
@@ -2432,7 +2432,7 @@
     <row r="105">
       <c r="C105" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
@@ -2453,7 +2453,7 @@
     <row r="106">
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
@@ -2474,7 +2474,7 @@
     <row r="107">
       <c r="C107" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
@@ -2495,7 +2495,7 @@
     <row r="108">
       <c r="C108" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
@@ -2516,7 +2516,7 @@
     <row r="109">
       <c r="C109" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="110">
       <c r="C110" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
@@ -2558,7 +2558,7 @@
     <row r="111">
       <c r="C111" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
@@ -2579,7 +2579,7 @@
     <row r="112">
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
@@ -2600,7 +2600,7 @@
     <row r="113">
       <c r="C113" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
@@ -2621,7 +2621,7 @@
     <row r="114">
       <c r="C114" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
@@ -2642,7 +2642,7 @@
     <row r="115">
       <c r="C115" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
@@ -2663,7 +2663,7 @@
     <row r="116">
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
@@ -2684,7 +2684,7 @@
     <row r="117">
       <c r="C117" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
@@ -2705,7 +2705,7 @@
     <row r="118">
       <c r="C118" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
@@ -2726,7 +2726,7 @@
     <row r="119">
       <c r="C119" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="120">
       <c r="C120" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
@@ -2768,7 +2768,7 @@
     <row r="121">
       <c r="C121" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
@@ -2789,7 +2789,7 @@
     <row r="122">
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
@@ -2810,7 +2810,7 @@
     <row r="123">
       <c r="C123" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
@@ -2831,7 +2831,7 @@
     <row r="124">
       <c r="C124" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
@@ -2852,7 +2852,7 @@
     <row r="125">
       <c r="C125" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
@@ -2873,7 +2873,7 @@
     <row r="126">
       <c r="C126" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr">
@@ -2894,7 +2894,7 @@
     <row r="127">
       <c r="C127" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr">
@@ -2915,7 +2915,7 @@
     <row r="128">
       <c r="C128" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr">
@@ -2936,7 +2936,7 @@
     <row r="129">
       <c r="C129" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="130">
       <c r="C130" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr">
@@ -2978,7 +2978,7 @@
     <row r="131">
       <c r="C131" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
@@ -2999,7 +2999,7 @@
     <row r="132">
       <c r="C132" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
@@ -3020,7 +3020,7 @@
     <row r="133">
       <c r="C133" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
@@ -3041,7 +3041,7 @@
     <row r="134">
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
@@ -3062,7 +3062,7 @@
     <row r="135">
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
@@ -3083,7 +3083,7 @@
     <row r="136">
       <c r="C136" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
@@ -3104,7 +3104,7 @@
     <row r="137">
       <c r="C137" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
@@ -3125,7 +3125,7 @@
     <row r="138">
       <c r="C138" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="139">
       <c r="C139" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="140">
       <c r="C140" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr">
@@ -3188,7 +3188,7 @@
     <row r="141">
       <c r="C141" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr">
@@ -3209,7 +3209,7 @@
     <row r="142">
       <c r="C142" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D142" s="10" t="inlineStr">
@@ -3230,7 +3230,7 @@
     <row r="143">
       <c r="C143" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="144">
       <c r="C144" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D144" s="10" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="145">
       <c r="C145" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D145" s="10" t="inlineStr">
@@ -3293,7 +3293,7 @@
     <row r="146">
       <c r="C146" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D146" s="10" t="inlineStr">
@@ -3314,7 +3314,7 @@
     <row r="147">
       <c r="C147" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D147" s="10" t="inlineStr">
@@ -3335,7 +3335,7 @@
     <row r="148">
       <c r="C148" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D148" s="10" t="inlineStr">
@@ -3356,7 +3356,7 @@
     <row r="149">
       <c r="C149" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D149" s="10" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="150">
       <c r="C150" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D150" s="10" t="inlineStr">
@@ -3398,7 +3398,7 @@
     <row r="151">
       <c r="C151" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D151" s="10" t="inlineStr">
@@ -3419,7 +3419,7 @@
     <row r="152">
       <c r="C152" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D152" s="10" t="inlineStr">
@@ -3440,7 +3440,7 @@
     <row r="153">
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D153" s="10" t="inlineStr">
@@ -3461,7 +3461,7 @@
     <row r="154">
       <c r="C154" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D154" s="10" t="inlineStr">
@@ -3482,7 +3482,7 @@
     <row r="155">
       <c r="C155" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D155" s="10" t="inlineStr">
@@ -3503,7 +3503,7 @@
     <row r="156">
       <c r="C156" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D156" s="10" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="157">
       <c r="C157" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D157" s="10" t="inlineStr">
@@ -3545,7 +3545,7 @@
     <row r="158">
       <c r="C158" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D158" s="10" t="inlineStr">
@@ -3566,7 +3566,7 @@
     <row r="159">
       <c r="C159" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D159" s="10" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="160">
       <c r="C160" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D160" s="10" t="inlineStr">
@@ -3608,7 +3608,7 @@
     <row r="161">
       <c r="C161" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D161" s="10" t="inlineStr">
@@ -3629,7 +3629,7 @@
     <row r="162">
       <c r="C162" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D162" s="10" t="inlineStr">
@@ -3650,7 +3650,7 @@
     <row r="163">
       <c r="C163" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D163" s="10" t="inlineStr">
@@ -3671,7 +3671,7 @@
     <row r="164">
       <c r="C164" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D164" s="10" t="inlineStr">
@@ -3692,7 +3692,7 @@
     <row r="165">
       <c r="C165" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D165" s="10" t="inlineStr">
@@ -3713,7 +3713,7 @@
     <row r="166">
       <c r="C166" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D166" s="10" t="inlineStr">
@@ -3734,7 +3734,7 @@
     <row r="167">
       <c r="C167" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D167" s="10" t="inlineStr">
@@ -3755,7 +3755,7 @@
     <row r="168">
       <c r="C168" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D168" s="10" t="inlineStr">
@@ -3776,7 +3776,7 @@
     <row r="169">
       <c r="C169" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D169" s="10" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="170">
       <c r="C170" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D170" s="10" t="inlineStr">
@@ -3818,7 +3818,7 @@
     <row r="171">
       <c r="C171" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D171" s="10" t="inlineStr">
@@ -3839,7 +3839,7 @@
     <row r="172">
       <c r="C172" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D172" s="10" t="inlineStr">
@@ -3860,7 +3860,7 @@
     <row r="173">
       <c r="C173" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D173" s="10" t="inlineStr">
@@ -3881,7 +3881,7 @@
     <row r="174">
       <c r="C174" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D174" s="10" t="inlineStr">
@@ -3902,7 +3902,7 @@
     <row r="175">
       <c r="C175" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D175" s="10" t="inlineStr">
@@ -3923,7 +3923,7 @@
     <row r="176">
       <c r="C176" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D176" s="10" t="inlineStr">
@@ -3944,7 +3944,7 @@
     <row r="177">
       <c r="C177" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D177" s="10" t="inlineStr">
@@ -3965,7 +3965,7 @@
     <row r="178">
       <c r="C178" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D178" s="10" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="179">
       <c r="C179" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D179" s="10" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="180">
       <c r="C180" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D180" s="10" t="inlineStr">
@@ -4028,7 +4028,7 @@
     <row r="181">
       <c r="C181" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D181" s="10" t="inlineStr">
@@ -4049,7 +4049,7 @@
     <row r="182">
       <c r="C182" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D182" s="10" t="inlineStr">
@@ -4070,7 +4070,7 @@
     <row r="183">
       <c r="C183" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D183" s="10" t="inlineStr">
@@ -4091,7 +4091,7 @@
     <row r="184">
       <c r="C184" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D184" s="10" t="inlineStr">
@@ -4112,7 +4112,7 @@
     <row r="185">
       <c r="C185" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D185" s="10" t="inlineStr">
@@ -4133,7 +4133,7 @@
     <row r="186">
       <c r="C186" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D186" s="10" t="inlineStr">
@@ -4154,7 +4154,7 @@
     <row r="187">
       <c r="C187" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D187" s="10" t="inlineStr">
@@ -4175,7 +4175,7 @@
     <row r="188">
       <c r="C188" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D188" s="10" t="inlineStr">
@@ -4196,7 +4196,7 @@
     <row r="189">
       <c r="C189" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D189" s="10" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="190">
       <c r="C190" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D190" s="10" t="inlineStr">
@@ -4238,7 +4238,7 @@
     <row r="191">
       <c r="C191" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D191" s="10" t="inlineStr">
@@ -4259,7 +4259,7 @@
     <row r="192">
       <c r="C192" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D192" s="10" t="inlineStr">
@@ -4280,7 +4280,7 @@
     <row r="193">
       <c r="C193" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D193" s="10" t="inlineStr">
@@ -4301,7 +4301,7 @@
     <row r="194">
       <c r="C194" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D194" s="10" t="inlineStr">
@@ -4322,7 +4322,7 @@
     <row r="195">
       <c r="C195" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D195" s="10" t="inlineStr">
@@ -4343,7 +4343,7 @@
     <row r="196">
       <c r="C196" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D196" s="10" t="inlineStr">
@@ -4364,7 +4364,7 @@
     <row r="197">
       <c r="C197" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D197" s="10" t="inlineStr">
@@ -4385,7 +4385,7 @@
     <row r="198">
       <c r="C198" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D198" s="10" t="inlineStr">
@@ -4406,7 +4406,7 @@
     <row r="199">
       <c r="C199" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D199" s="10" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="200">
       <c r="C200" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D200" s="10" t="inlineStr">
@@ -4448,7 +4448,7 @@
     <row r="201">
       <c r="C201" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D201" s="10" t="inlineStr">
@@ -4469,7 +4469,7 @@
     <row r="202">
       <c r="C202" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D202" s="10" t="inlineStr">
@@ -4490,7 +4490,7 @@
     <row r="203">
       <c r="C203" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D203" s="10" t="inlineStr">
@@ -4511,7 +4511,7 @@
     <row r="204">
       <c r="C204" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D204" s="10" t="inlineStr">
@@ -4532,7 +4532,7 @@
     <row r="205">
       <c r="C205" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D205" s="10" t="inlineStr">
@@ -4553,7 +4553,7 @@
     <row r="206">
       <c r="C206" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D206" s="10" t="inlineStr">
@@ -4574,7 +4574,7 @@
     <row r="207">
       <c r="C207" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D207" s="10" t="inlineStr">
@@ -4595,7 +4595,7 @@
     <row r="208">
       <c r="C208" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D208" s="10" t="inlineStr">
@@ -4616,7 +4616,7 @@
     <row r="209">
       <c r="C209" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D209" s="10" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="210">
       <c r="C210" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D210" s="10" t="inlineStr">
@@ -4658,7 +4658,7 @@
     <row r="211">
       <c r="C211" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D211" s="10" t="inlineStr">
@@ -4679,7 +4679,7 @@
     <row r="212">
       <c r="C212" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D212" s="10" t="inlineStr">
@@ -4700,7 +4700,7 @@
     <row r="213">
       <c r="C213" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D213" s="10" t="inlineStr">
@@ -4721,7 +4721,7 @@
     <row r="214">
       <c r="C214" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D214" s="10" t="inlineStr">
@@ -4742,7 +4742,7 @@
     <row r="215">
       <c r="C215" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D215" s="10" t="inlineStr">
@@ -4763,7 +4763,7 @@
     <row r="216">
       <c r="C216" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D216" s="10" t="inlineStr">
@@ -4784,7 +4784,7 @@
     <row r="217">
       <c r="C217" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D217" s="10" t="inlineStr">
@@ -4805,7 +4805,7 @@
     <row r="218">
       <c r="C218" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D218" s="10" t="inlineStr">
@@ -4826,7 +4826,7 @@
     <row r="219">
       <c r="C219" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D219" s="10" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="220">
       <c r="C220" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D220" s="10" t="inlineStr">
@@ -4868,7 +4868,7 @@
     <row r="221">
       <c r="C221" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D221" s="10" t="inlineStr">
@@ -4889,7 +4889,7 @@
     <row r="222">
       <c r="C222" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D222" s="10" t="inlineStr">
@@ -4910,7 +4910,7 @@
     <row r="223">
       <c r="C223" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D223" s="10" t="inlineStr">
@@ -4931,7 +4931,7 @@
     <row r="224">
       <c r="C224" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D224" s="10" t="inlineStr">
@@ -4952,7 +4952,7 @@
     <row r="225">
       <c r="C225" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D225" s="10" t="inlineStr">
@@ -4973,7 +4973,7 @@
     <row r="226">
       <c r="C226" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D226" s="10" t="inlineStr">
@@ -4994,7 +4994,7 @@
     <row r="227">
       <c r="C227" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D227" s="10" t="inlineStr">
@@ -5015,7 +5015,7 @@
     <row r="228">
       <c r="C228" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D228" s="10" t="inlineStr">
@@ -5036,7 +5036,7 @@
     <row r="229">
       <c r="C229" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D229" s="10" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="230">
       <c r="C230" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D230" s="10" t="inlineStr">
@@ -5078,7 +5078,7 @@
     <row r="231">
       <c r="C231" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D231" s="10" t="inlineStr">
@@ -5099,7 +5099,7 @@
     <row r="232">
       <c r="C232" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D232" s="10" t="inlineStr">
@@ -5120,7 +5120,7 @@
     <row r="233">
       <c r="C233" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D233" s="10" t="inlineStr">
@@ -5141,7 +5141,7 @@
     <row r="234">
       <c r="C234" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D234" s="10" t="inlineStr">
@@ -5162,7 +5162,7 @@
     <row r="235">
       <c r="C235" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D235" s="10" t="inlineStr">
@@ -5183,7 +5183,7 @@
     <row r="236">
       <c r="C236" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D236" s="10" t="inlineStr">
@@ -5204,7 +5204,7 @@
     <row r="237">
       <c r="C237" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D237" s="10" t="inlineStr">
@@ -5225,7 +5225,7 @@
     <row r="238">
       <c r="C238" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D238" s="10" t="inlineStr">
@@ -5246,7 +5246,7 @@
     <row r="239">
       <c r="C239" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D239" s="10" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="240">
       <c r="C240" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D240" s="10" t="inlineStr">
@@ -5288,7 +5288,7 @@
     <row r="241">
       <c r="C241" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D241" s="10" t="inlineStr">
@@ -5309,7 +5309,7 @@
     <row r="242">
       <c r="C242" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D242" s="10" t="inlineStr">
@@ -5330,7 +5330,7 @@
     <row r="243">
       <c r="C243" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D243" s="10" t="inlineStr">
@@ -5351,7 +5351,7 @@
     <row r="244">
       <c r="C244" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D244" s="10" t="inlineStr">
@@ -5372,7 +5372,7 @@
     <row r="245">
       <c r="C245" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D245" s="10" t="inlineStr">
@@ -5393,7 +5393,7 @@
     <row r="246">
       <c r="C246" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D246" s="10" t="inlineStr">
@@ -5414,7 +5414,7 @@
     <row r="247">
       <c r="C247" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D247" s="10" t="inlineStr">
@@ -5435,7 +5435,7 @@
     <row r="248">
       <c r="C248" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>FACTURA PROVEEDOR</t>
         </is>
       </c>
       <c r="D248" s="10" t="inlineStr">
@@ -7606,59 +7606,26 @@
       </c>
       <c r="D314" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Costo de Transferen</t>
         </is>
       </c>
       <c r="E314" s="6" t="n">
-        <v>151.3599999413127</v>
+        <v>-3000</v>
       </c>
       <c r="F314" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Costo de Transferen</t>
         </is>
       </c>
       <c r="G314" s="10" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>WOB</t>
         </is>
       </c>
       <c r="H314" s="6" t="n">
-        <v>151.3599999413127</v>
+        <v>-3000</v>
       </c>
       <c r="I314" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="315">
-      <c r="C315" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos no asociados a FC</t>
-        </is>
-      </c>
-      <c r="D315" s="10" t="inlineStr">
-        <is>
-          <t>Costo de Transferen</t>
-        </is>
-      </c>
-      <c r="E315" s="6" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F315" s="10" t="inlineStr">
-        <is>
-          <t>Costo de Transferen</t>
-        </is>
-      </c>
-      <c r="G315" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H315" s="6" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="I315" s="11" t="inlineStr">
         <is>
           <t>MENORES VALORES</t>
         </is>

</xml_diff>